<commit_message>
Wire scripts and docs to organized layout
</commit_message>
<xml_diff>
--- a/outputs/signed_up/techweek_signed_up_transport_schedule.xlsx
+++ b/outputs/signed_up/techweek_signed_up_transport_schedule.xlsx
@@ -123,20 +123,25 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
+          <t xml:space="preserve">sales_coaching</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t xml:space="preserve">rank</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t xml:space="preserve">tier</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t xml:space="preserve">opportunity_score</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t xml:space="preserve">event_url</t>
         </is>
@@ -270,6 +275,11 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/FHiuNwzr13e3YBI4ssUX</t>
         </is>
       </c>
@@ -387,20 +397,30 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use the agent/spec theme. Say you are studying how specs, PRs, and Slack context survive agentic workflows.
+Ask: When an agent touches a ticket, what artifact proves who shaped the outcome?
+Listen for: Specs as source of truth, issue quality, review quality, manager trust, missing context.
+Follow-up: Ask for 20 minutes with whoever owns engineering process or agent adoption.</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
           <t xml:space="preserve">24</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t xml:space="preserve">74</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/FHiuNwzr13e3YBI4ssUX</t>
         </is>
@@ -534,6 +554,11 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/xowd9F3kB7mPFN1luUwY</t>
         </is>
       </c>
@@ -651,20 +676,30 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Frame vibe coding as a team-process problem, not a solo productivity trick.
+Ask: What breaks when vibe coding becomes team development across reviews, specs, and handoffs?
+Listen for: Review bottlenecks, low-trust AI output, unclear ownership, managers losing visibility.
+Follow-up: Send a short write-up on contribution evidence for AI-assisted teams.</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
           <t xml:space="preserve">29</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t xml:space="preserve">71</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/xowd9F3kB7mPFN1luUwY</t>
         </is>
@@ -783,20 +818,30 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use the Slack angle: work decisions often happen outside GitHub.
+Ask: Which important engineering decisions live in Slack, and do they ever make it into reviews or planning?
+Listen for: Slack decisions, cross-functional handoffs, lost context, collaboration evidence.
+Follow-up: Ask whether Slack-linked contribution credit would help managers or team leads.</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
           <t xml:space="preserve">180</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t xml:space="preserve">53</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/dmFBKIxzn2LdFmktqas8</t>
         </is>
@@ -930,6 +975,11 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/OF1vP5L8dtXKRtInyWKs?c=s6u4EYds</t>
         </is>
       </c>
@@ -1047,20 +1097,30 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Hardware and robotics teams have heavy coordination work before code ships.
+Ask: How do you credit specs, integration debugging, reviews, and ops work across hardware/software boundaries?
+Listen for: Systems integration, test evidence, field debugging, cross-discipline ownership.
+Follow-up: Ask for founder/operator feedback rather than pushing a pure software-team sale.</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
           <t xml:space="preserve">13</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t xml:space="preserve">86</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/09a0qPKv0cSOIOSGxjTQ</t>
         </is>
@@ -1179,20 +1239,30 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Open-source rooms should hear the maintainer-labor angle first.
+Ask: How do you credit review, triage, specs, and maintainer work that never becomes a commit?
+Listen for: Contributor rewards, bounty systems, maintainer burnout, attribution disputes.
+Follow-up: Ask for intros to maintainers, DevRel leads, or teams running contributor programs.</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
           <t xml:space="preserve">37</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t xml:space="preserve">64</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/OF1vP5L8dtXKRtInyWKs?c=s6u4EYds</t>
         </is>
@@ -1311,20 +1381,30 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This is broad B2B. Keep the pitch short and qualify fast.
+Ask: Does your engineering team use GitHub and Slack heavily enough that contribution visibility is a management problem?
+Listen for: Founder with 5+ engineers, remote team, AI coding adoption, performance-review pain.
+Follow-up: Ask for a warm intro to the CTO or VP Eng if the person is not the buyer.</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
           <t xml:space="preserve">169</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t xml:space="preserve">54</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/oQvmxTsHOVayx47ok3li?c=0hT1WkMm</t>
         </is>
@@ -1458,6 +1538,11 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/OF1vP5L8dtXKRtInyWKs?c=s6u4EYds</t>
         </is>
       </c>
@@ -1590,6 +1675,11 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/M7pXmV8sOXT11yHb9pKw</t>
         </is>
       </c>
@@ -1707,20 +1797,30 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use enterprise SDLC language: trustworthy artifacts, change control, and evidence trails.
+Ask: Which engineering artifacts stay reliable when AI changes how teams plan, review, and ship?
+Listen for: Auditability, manager reports, PR review evidence, specs scattered across tools.
+Follow-up: Ask to compare their SDLC reporting process with an Accolades evidence report.</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
           <t xml:space="preserve">33</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t xml:space="preserve">68</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/M7pXmV8sOXT11yHb9pKw</t>
         </is>
@@ -1839,20 +1939,30 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: For MCP/control-plane conversations, talk about instrumenting context and actions.
+Ask: What needs to be logged so a manager can understand who influenced an agent-driven outcome?
+Listen for: Context sources, tool permissions, traceability, review responsibility, platform ownership.
+Follow-up: Ask to compare notes with anyone building internal agent infrastructure.</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
           <t xml:space="preserve">7</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t xml:space="preserve">98</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="AA14" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/5vHvRPI0VlMQwOmQadCN</t>
         </is>
@@ -1971,20 +2081,30 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This is the highest-priority CTO/platform room. Lead with the control-plane problem.
+Ask: What should managers measure once copilots are part of every development workflow?
+Listen for: CTO/VP Eng pain, platform ownership, productivity reporting, GitHub/code review evidence.
+Follow-up: Push for a concrete post-Tech Week call if they own DevEx, platform, or engineering metrics.</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t xml:space="preserve">100</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/bn5h1g13xzOV6R5XkLaE</t>
         </is>
@@ -2103,20 +2223,30 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: API and identity demos are a good opening for permissions plus evidence.
+Ask: When agents call internal APIs, how do you audit who requested, reviewed, and approved the work?
+Listen for: API governance, permissions, review evidence, enterprise buyers, workflow logs.
+Follow-up: Ask for intros to teams responsible for developer platform or internal API governance.</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
           <t xml:space="preserve">217</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t xml:space="preserve">51</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/XqIBMZmB4oubCZWFP2Sl</t>
         </is>
@@ -2235,20 +2365,30 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use liability language carefully: evidence, review, and accountability.
+Ask: If AI-assisted work causes a problem, what evidence would you want before assigning responsibility?
+Listen for: Audit trails, legal/compliance sensitivity, review records, decision provenance.
+Follow-up: Ask if source-linked engineering evidence would be useful for compliance conversations.</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
           <t xml:space="preserve">72</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t xml:space="preserve">58</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/UBrZopzqpRwbn6Qk0npO?c=4IfpVNvT</t>
         </is>
@@ -2382,6 +2522,11 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/7DYGSiY1WUuRSvEnD5gp?c=aQ_TnSt9</t>
         </is>
       </c>
@@ -2499,20 +2644,30 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Enterprise AI buyers care about governance and platform ownership.
+Ask: Where do manager reports and audit evidence fit into your enterprise AI rollout?
+Listen for: Governance, internal platforms, production agents, executive reporting, risk controls.
+Follow-up: Ask for a specific post-event call with the platform, DevEx, or AI governance owner.</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="Y19" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="Z19" t="inlineStr">
         <is>
           <t xml:space="preserve">100</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="AA19" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/FSzOO6xPn11iqxVdtQ9j?</t>
         </is>
@@ -2631,20 +2786,30 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use infrastructure scale as the bridge into contribution evidence.
+Ask: In the agent era, what evidence do infra teams need to trust work done across tools and systems?
+Listen for: Platform scale, agent infrastructure, toolchain visibility, engineering productivity.
+Follow-up: Ask for technical feedback from infra leaders rather than a generic founder follow-up.</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
           <t xml:space="preserve">23</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="Z20" t="inlineStr">
         <is>
           <t xml:space="preserve">75</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="AA20" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/jytNb4IdG0HxwJnqDSgf</t>
         </is>
@@ -2763,20 +2928,30 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use DevEx language and avoid sounding like HR analytics.
+Ask: Where does DevEx stop being tooling and start being contribution evidence?
+Listen for: Internal developer platforms, friction measurement, review quality, invisible glue work.
+Follow-up: Ask who owns DevEx metrics and whether source-linked contribution evidence would help.</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
           <t xml:space="preserve">3</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="Z21" t="inlineStr">
         <is>
           <t xml:space="preserve">100</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/7DYGSiY1WUuRSvEnD5gp?c=aQ_TnSt9</t>
         </is>
@@ -2910,6 +3085,11 @@
       </c>
       <c r="Z22" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/7DYGSiY1WUuRSvEnD5gp?c=aQ_TnSt9</t>
         </is>
       </c>
@@ -3042,6 +3222,11 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/4HvzWY1VZlHgK21fMBUz?c=g5NbnbjN</t>
         </is>
       </c>
@@ -3159,20 +3344,30 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Tie security and data controls to audit-ready engineering evidence.
+Ask: How are you proving AI-assisted engineering work was reviewed without leaking sensitive context?
+Listen for: Security reviews, data access, compliance needs, audit trails, manager sign-off.
+Follow-up: Offer a follow-up focused on source-linked evidence without surveillance dashboards.</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
           <t xml:space="preserve">16</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="Z24" t="inlineStr">
         <is>
           <t xml:space="preserve">80</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/4HvzWY1VZlHgK21fMBUz?c=g5NbnbjN</t>
         </is>
@@ -3291,20 +3486,30 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: AI-native founders will understand the operating-model shift.
+Ask: How do AI-native teams evaluate human contribution when agents produce more of the visible output?
+Listen for: Small teams scaling fast, agent-heavy workflows, contribution rewards, manager memory breaking down.
+Follow-up: Ask for a founder-to-founder product critique and one relevant buyer intro.</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
           <t xml:space="preserve">9</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="Y25" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="Z25" t="inlineStr">
         <is>
           <t xml:space="preserve">94</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="AA25" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/titPml1Nw0DKwGl9B6CF</t>
         </is>
@@ -3438,6 +3643,11 @@
       </c>
       <c r="Z26" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/1N6CtiCpYquktoTh5NUm</t>
         </is>
       </c>
@@ -3555,20 +3765,30 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Talk about the IDE as the point where human and agent work blur.
+Ask: When agents write code, what human work still needs credit?
+Listen for: Prompting, spec writing, review corrections, architectural judgment, tool orchestration.
+Follow-up: Ask to sanity-check the Accolades framing with builders using coding agents daily.</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
           <t xml:space="preserve">27</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="Y27" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
+      <c r="Z27" t="inlineStr">
         <is>
           <t xml:space="preserve">72</t>
         </is>
       </c>
-      <c r="Z27" t="inlineStr">
+      <c r="AA27" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/1N6CtiCpYquktoTh5NUm</t>
         </is>
@@ -3702,6 +3922,11 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/E8NhJNHWGhMetLlrFvQ7</t>
         </is>
       </c>
@@ -3819,20 +4044,30 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Agent harnesses are about production reliability; connect that to human accountability.
+Ask: What human evidence needs to sit beside the harness output before an enterprise trusts agent work?
+Listen for: Enterprise adoption, internal platforms, review gates, evaluation records, ownership.
+Follow-up: Ask to discuss how Accolades could consume evidence from agent harness workflows.</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
           <t xml:space="preserve">8</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="Y29" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
+      <c r="Z29" t="inlineStr">
         <is>
           <t xml:space="preserve">97</t>
         </is>
       </c>
-      <c r="Z29" t="inlineStr">
+      <c r="AA29" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/2NP0rZW8BmdGAGUOEhGP?f=1</t>
         </is>
@@ -3951,20 +4186,30 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use the event title directly: if agents are users, the system of record matters.
+Ask: If the agent is the user, what becomes the system of record for useful work?
+Listen for: Tool schemas, docs, prompts, guardrails, review evidence, ownership boundaries.
+Follow-up: Ask for feedback on whether Accolades should track agent-orchestration evidence explicitly.</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
           <t xml:space="preserve">15</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
+      <c r="Y30" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y30" t="inlineStr">
+      <c r="Z30" t="inlineStr">
         <is>
           <t xml:space="preserve">81</t>
         </is>
       </c>
-      <c r="Z30" t="inlineStr">
+      <c r="AA30" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/E8NhJNHWGhMetLlrFvQ7</t>
         </is>
@@ -4003,7 +4248,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">applied</t>
+          <t xml:space="preserve">registered</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -4033,7 +4278,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">[TW-4778] [PENDING CURATED] The CTO Mixer: Humanizing Tech | Happy Hour</t>
+          <t xml:space="preserve">[TW-4778] [REG CURATED] The CTO Mixer: Humanizing Tech | Happy Hour</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -4078,25 +4323,35 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wait for host approval Submitted via Partiful API; rsvpStatus=PENDING_APPROVAL; count=1; plusOne=none.</t>
+          <t xml:space="preserve">On the list; monitor for updates Partiful page shows ON THE LIST as of 2026-05-10. Previously submitted via Partiful API; rsvpStatus=PENDING_APPROVAL; count=1; plusOne=none.</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This is a direct CTO room. Ask about pain before explaining the product.
+Ask: What is hardest for your managers to evaluate now that AI touches more engineering work?
+Listen for: Performance reviews, planning evidence, PR quality, distributed-team context, DevEx ownership.
+Follow-up: If pain is clear, ask for a 20-minute CTO follow-up and permission to send a one-pager.</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
           <t xml:space="preserve">6</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr">
+      <c r="Y31" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y31" t="inlineStr">
+      <c r="Z31" t="inlineStr">
         <is>
           <t xml:space="preserve">100</t>
         </is>
       </c>
-      <c r="Z31" t="inlineStr">
+      <c r="AA31" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/h1hGv0PkskcagJOv5M9K</t>
         </is>
@@ -4215,20 +4470,30 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Keep this practical: agents at work means work attribution is getting messy.
+Ask: When an agent helps ship something, who gets credit for the useful parts of the workflow?
+Listen for: Agent orchestration, prompt/spec work, review corrections, workflow ownership.
+Follow-up: Ask for examples of workflows Accolades should recognize or avoid recognizing.</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
           <t xml:space="preserve">19</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
+      <c r="Y32" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
+      <c r="Z32" t="inlineStr">
         <is>
           <t xml:space="preserve">78</t>
         </is>
       </c>
-      <c r="Z32" t="inlineStr">
+      <c r="AA32" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/Fp5STyPH0McEt0awlWFD</t>
         </is>
@@ -4362,6 +4627,11 @@
       </c>
       <c r="Z33" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/events/6ZuudQBBZXcMNjdMynJ2</t>
         </is>
       </c>
@@ -4479,20 +4749,30 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: MCP people will understand context plumbing. Map that to later evaluation.
+Ask: What context should tools expose so contribution can be evaluated after the work ships?
+Listen for: Tool-call trails, context sources, agent actions, human review, integration ownership.
+Follow-up: Ask for technical feedback on evidence capture from tool and agent workflows.</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
           <t xml:space="preserve">58</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
+      <c r="Y34" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y34" t="inlineStr">
+      <c r="Z34" t="inlineStr">
         <is>
           <t xml:space="preserve">63</t>
         </is>
       </c>
-      <c r="Z34" t="inlineStr">
+      <c r="AA34" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/events/6ZuudQBBZXcMNjdMynJ2</t>
         </is>
@@ -4611,20 +4891,30 @@
       </c>
       <c r="W35" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use leadership language: visibility without surveillance.
+Ask: What evidence do tech leaders wish they had for planning and reviews without turning into surveillance?
+Listen for: Manager reporting, trust, team health, engineering productivity, executive visibility.
+Follow-up: Ask for a leadership-focused follow-up if they manage engineers or internal platforms.</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
           <t xml:space="preserve">5</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
+      <c r="Y35" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y35" t="inlineStr">
+      <c r="Z35" t="inlineStr">
         <is>
           <t xml:space="preserve">100</t>
         </is>
       </c>
-      <c r="Z35" t="inlineStr">
+      <c r="AA35" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/UhyErPPxuo2vELIutdGj?</t>
         </is>
@@ -4758,6 +5048,11 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/events/6ZuudQBBZXcMNjdMynJ2</t>
         </is>
       </c>
@@ -4890,6 +5185,11 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/5K5c4eODrGPKME7or20H</t>
         </is>
       </c>
@@ -5007,20 +5307,30 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This is a direct AI-coding workflow room. Start with manager trust.
+Ask: What changed in your review process after AI started writing more code?
+Listen for: Review overload, shallow approvals, unclear ownership, productivity claims without evidence.
+Follow-up: Ask for a buyer call with the engineering leader responsible for AI coding adoption.</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
           <t xml:space="preserve">4</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
+      <c r="Y38" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y38" t="inlineStr">
+      <c r="Z38" t="inlineStr">
         <is>
           <t xml:space="preserve">100</t>
         </is>
       </c>
-      <c r="Z38" t="inlineStr">
+      <c r="AA38" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/5K5c4eODrGPKME7or20H</t>
         </is>
@@ -5139,20 +5449,30 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: For agent scale, focus on attribution across many automated steps.
+Ask: When agents run at scale, how do you separate valuable human judgment from automated output?
+Listen for: Evaluation gaps, agent ops, review ownership, platform labor, traceability.
+Follow-up: Ask to learn how they log agent work today and whether source-linked credit would fit.</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
           <t xml:space="preserve">10</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
+      <c r="Y39" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y39" t="inlineStr">
+      <c r="Z39" t="inlineStr">
         <is>
           <t xml:space="preserve">93</t>
         </is>
       </c>
-      <c r="Z39" t="inlineStr">
+      <c r="AA39" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/6BlGFmwIdpyndqyLYS2v?c=bv5YqCoL</t>
         </is>
@@ -5271,20 +5591,30 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This is a live-demo room. Use your own build story, then ask about workflow data.
+Ask: Which parts of your AI workflow create useful evidence that managers should see later?
+Listen for: Prompting, issue specs, PRs, Slack decisions, demos that could become repeatable workflows.
+Follow-up: Ask demo builders to name one evidence source Accolades should integrate first.</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
           <t xml:space="preserve">34</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
+      <c r="Y40" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y40" t="inlineStr">
+      <c r="Z40" t="inlineStr">
         <is>
           <t xml:space="preserve">66</t>
         </is>
       </c>
-      <c r="Z40" t="inlineStr">
+      <c r="AA40" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/sGvp4VIr3KrGqRoWCKhV</t>
         </is>
@@ -5403,20 +5733,30 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This may be the best direct engineering-manager room. Be crisp and buyer-oriented.
+Ask: What do your managers use as evidence when deciding who moved a project forward?
+Listen for: Performance-review pain, review quality, planning work, manager memory, team rewards.
+Follow-up: Ask for a concrete follow-up with the engineering leader or manager who owns the pain.</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
           <t xml:space="preserve">20</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
+      <c r="Y41" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y41" t="inlineStr">
+      <c r="Z41" t="inlineStr">
         <is>
           <t xml:space="preserve">78</t>
         </is>
       </c>
-      <c r="Z41" t="inlineStr">
+      <c r="AA41" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/bETmU06uq4TtORng6I1l</t>
         </is>
@@ -5550,6 +5890,11 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/X0u5GrmzvIUTrjoAOgVm</t>
         </is>
       </c>
@@ -5667,20 +6012,30 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: This is less direct; use prediction and decision quality as the bridge.
+Ask: How do you know which people or artifacts actually improved a technical decision?
+Listen for: Decision provenance, forecasts versus outcomes, accountability, source-linked context.
+Follow-up: Only pursue deep follow-up if they have an engineering team with GitHub/Slack pain.</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
           <t xml:space="preserve">89</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr">
+      <c r="Y43" t="inlineStr">
         <is>
           <t xml:space="preserve">B</t>
         </is>
       </c>
-      <c r="Y43" t="inlineStr">
+      <c r="Z43" t="inlineStr">
         <is>
           <t xml:space="preserve">57</t>
         </is>
       </c>
-      <c r="Z43" t="inlineStr">
+      <c r="AA43" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/eSldi3iNIvAVo9utdd8S</t>
         </is>
@@ -5799,20 +6154,30 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: At dinner, sell softly. Use founder-to-founder learning first.
+Ask: How are AI builders changing how they reward and evaluate work inside their teams?
+Listen for: AI-native operating models, fast-growing teams, founder pain, engineering leadership gaps.
+Follow-up: Ask for one sharp product critique and one relevant engineering-leader intro.</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
           <t xml:space="preserve">11</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr">
+      <c r="Y44" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y44" t="inlineStr">
+      <c r="Z44" t="inlineStr">
         <is>
           <t xml:space="preserve">90</t>
         </is>
       </c>
-      <c r="Z44" t="inlineStr">
+      <c r="AA44" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/idltitmjA4ZzL9IuK0Y6</t>
         </is>
@@ -5931,20 +6296,30 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use the codebase-as-spec theme and make Accolades feel complementary.
+Ask: What would make a codebase trustworthy enough for agents and managers?
+Listen for: Source-linked context, specs in code, review trails, stale docs, manager confidence.
+Follow-up: Ask to exchange notes on codebase evidence and Accolades after the event.</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
           <t xml:space="preserve">21</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr">
+      <c r="Y45" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y45" t="inlineStr">
+      <c r="Z45" t="inlineStr">
         <is>
           <t xml:space="preserve">76</t>
         </is>
       </c>
-      <c r="Z45" t="inlineStr">
+      <c r="AA45" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/X0u5GrmzvIUTrjoAOgVm</t>
         </is>
@@ -6063,20 +6438,30 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Use the DM/agent framing to talk about decisions in conversational channels.
+Ask: When agents and teammates work in DMs, what context should be preserved for later credit or audit?
+Listen for: Slack/DM work, agent conversations, missing provenance, informal decisions.
+Follow-up: Ask for feedback on Slack-first evidence capture if the person runs engineering workflows.</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr">
+      <c r="Y46" t="inlineStr">
         <is>
           <t xml:space="preserve">S</t>
         </is>
       </c>
-      <c r="Y46" t="inlineStr">
+      <c r="Z46" t="inlineStr">
         <is>
           <t xml:space="preserve">79</t>
         </is>
       </c>
-      <c r="Z46" t="inlineStr">
+      <c r="AA46" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/ed2EFWip0do9OuYmVPZI</t>
         </is>
@@ -6210,6 +6595,11 @@
       </c>
       <c r="Z47" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/X0u5GrmzvIUTrjoAOgVm</t>
         </is>
       </c>
@@ -6342,6 +6732,11 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/jkjGahQgmH9PLIxjfTFt</t>
         </is>
       </c>
@@ -6459,20 +6854,30 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: For agent fleet and autonomous systems people, focus on orchestration accountability.
+Ask: How do teams know who did useful orchestration, review, and correction work across agent fleets?
+Listen for: Multi-agent coordination, operations work, incident reviews, hidden platform labor.
+Follow-up: Ask for intros to platform leads running agent or automation infrastructure.</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
           <t xml:space="preserve">45</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr">
+      <c r="Y49" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y49" t="inlineStr">
+      <c r="Z49" t="inlineStr">
         <is>
           <t xml:space="preserve">64</t>
         </is>
       </c>
-      <c r="Z49" t="inlineStr">
+      <c r="AA49" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/jkjGahQgmH9PLIxjfTFt</t>
         </is>
@@ -6591,20 +6996,30 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sales coaching:
+Pitch: Accolades credits the engineering work commit counts miss, using source-linked GitHub and Slack evidence.
+Open: Treat this as a lower-pressure builder salon and look for AI-native founders.
+Ask: How does your team credit prompt work, specs, review, and product judgment around AI coding?
+Listen for: Builder workflows, early team habits, contribution rewards, technical-founder pain.
+Follow-up: Ask for feedback or an intro; do not over-invest unless they match the ICP.</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
           <t xml:space="preserve">26</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
+      <c r="Y50" t="inlineStr">
         <is>
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="Y50" t="inlineStr">
+      <c r="Z50" t="inlineStr">
         <is>
           <t xml:space="preserve">73</t>
         </is>
       </c>
-      <c r="Z50" t="inlineStr">
+      <c r="AA50" t="inlineStr">
         <is>
           <t xml:space="preserve">https://partiful.com/e/kvGpuFMeACW7ZWPYtxTP</t>
         </is>
@@ -6738,11 +7153,16 @@
       </c>
       <c r="Z51" t="inlineStr">
         <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://partiful.com/e/jkjGahQgmH9PLIxjfTFt</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z51"/>
+  <autoFilter ref="A1:AA51"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix agent markdown rendering and deploy flow
</commit_message>
<xml_diff>
--- a/outputs/signed_up/techweek_signed_up_transport_schedule.xlsx
+++ b/outputs/signed_up/techweek_signed_up_transport_schedule.xlsx
@@ -798,12 +798,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Bryant Park, New York, NY</t>
+          <t>Boucherie, 145 W 53rd St, New York, NY</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>approx_from_calendar_location</t>
+          <t>exact_from_signup_status</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Bryant+Park%2C+New+York%2C+NY</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Boucherie%2C+145+W+53rd+St%2C+New+York%2C+NY</t>
         </is>
       </c>
     </row>
@@ -6426,12 +6426,12 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Spring St and Broadway, New York, NY</t>
+          <t>Rockefeller Center, New York, NY</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>approx_from_calendar_location</t>
+          <t>approx_from_signup_status</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Spring+St+and+Broadway%2C+New+York%2C+NY</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rockefeller+Center%2C+New+York%2C+NY</t>
         </is>
       </c>
     </row>
@@ -6710,12 +6710,12 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>23rd Street and Broadway, New York, NY</t>
+          <t>ilili, 236 5th Ave, New York, NY</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>approx_from_calendar_location</t>
+          <t>exact_from_signup_status</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=23rd+Street+and+Broadway%2C+New+York%2C+NY</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=ilili%2C+236+5th+Ave%2C+New+York%2C+NY</t>
         </is>
       </c>
     </row>
@@ -7146,12 +7146,12 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Central Park, Manhattan, NY</t>
+          <t>Central Park, Manhattan, New York, NY</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>approx_from_calendar_location</t>
+          <t>approx_from_signup_status</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -7211,7 +7211,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Central+Park%2C+Manhattan%2C+NY</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Central+Park%2C+Manhattan%2C+New+York%2C+NY</t>
         </is>
       </c>
     </row>
@@ -7288,12 +7288,12 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Spring St and Broadway, New York, NY</t>
+          <t>1/2 Bond St, 1 Bond St, New York, NY</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>approx_from_calendar_location</t>
+          <t>exact_from_signup_status</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Spring+St+and+Broadway%2C+New+York%2C+NY</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=1%2F2+Bond+St%2C+1+Bond+St%2C+New+York%2C+NY</t>
         </is>
       </c>
     </row>
@@ -8120,7 +8120,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-06-04 11:59</t>
+          <t>2026-06-04 11:43</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>2026-06-04 11:59</t>
+          <t>2026-06-04 11:43</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -8165,17 +8165,17 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>47</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Walk 3 min to Fulton St (2/3); subway 22 min; walk 1 min from 28 St (N/Q/R/W); includes 5 min buffer.</t>
+          <t>Walk 3 min to Fulton St (2/3); subway 35 min; walk 4 min from 5 Av/53 St (E/F); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>2 Fulton St to 28 St</t>
+          <t>2 Fulton St to 50 St; E 50 St to 5 Av/53 St</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -8215,7 +8215,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=40.7084297%2C-74.0056635&amp;destination=40.7458%2C-73.9888&amp;travelmode=transit</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=40.7084297%2C-74.0056635&amp;destination=40.7598219%2C-73.9724708&amp;travelmode=transit</t>
         </is>
       </c>
     </row>
@@ -8292,12 +8292,12 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>28th Street and Broadway, New York, NY</t>
+          <t>Midtown East, New York, NY</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>approx_from_calendar_location</t>
+          <t>approx_from_signup_status</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=28th+Street+and+Broadway%2C+New+York%2C+NY</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Midtown+East%2C+New+York%2C+NY</t>
         </is>
       </c>
     </row>
@@ -8688,7 +8688,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-06-04 15:46</t>
+          <t>2026-06-04 15:10</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>2026-06-04 15:46</t>
+          <t>2026-06-04 15:10</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -8733,22 +8733,22 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>50</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Walk 1 min to 28 St (N/Q/R/W); subway 6 min; walk 2 min from 8 St-NYU (N/Q/R/W); includes 5 min buffer.</t>
+          <t>Walk 4 min to 5 Av/53 St (E/F); subway 39 min; walk 2 min from 8 St-NYU (N/Q/R/W); includes 5 min buffer.</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>N 28 St to 8 St-NYU</t>
+          <t>E 5 Av/53 St to Woodhaven Blvd; R Woodhaven Blvd to 8 St-NYU</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>Normal service</t>
+          <t>Minor delays possible</t>
         </is>
       </c>
       <c r="V61" t="inlineStr">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=40.7458%2C-73.9888&amp;destination=40.729391%2C-73.9921562&amp;travelmode=transit</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=40.7598219%2C-73.9724708&amp;destination=40.729391%2C-73.9921562&amp;travelmode=transit</t>
         </is>
       </c>
     </row>

</xml_diff>